<commit_message>
Restrict Sales Order Creation for Rejected/Suspended Agent
</commit_message>
<xml_diff>
--- a/Documents/Prouct_List_V2_new.xlsx
+++ b/Documents/Prouct_List_V2_new.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\SuperCRM\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7476CFCB-3C26-4346-B3B8-77B72EE410B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7635"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -440,7 +441,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -864,37 +865,37 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
-    <col min="2" max="2" width="37.5703125" customWidth="1"/>
+    <col min="2" max="2" width="37.54296875" customWidth="1"/>
     <col min="3" max="3" width="39" customWidth="1"/>
-    <col min="4" max="4" width="47.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="55.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="65.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="75.140625" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.7109375" customWidth="1"/>
-    <col min="14" max="14" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="21.42578125" customWidth="1"/>
-    <col min="19" max="19" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="26.85546875" customWidth="1"/>
-    <col min="21" max="21" width="27.28515625" customWidth="1"/>
-    <col min="22" max="22" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="14.42578125" customWidth="1"/>
-    <col min="24" max="24" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="47.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="65.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.26953125" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" customWidth="1"/>
+    <col min="9" max="9" width="75.1796875" customWidth="1"/>
+    <col min="10" max="10" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.54296875" customWidth="1"/>
+    <col min="12" max="12" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.7265625" customWidth="1"/>
+    <col min="14" max="14" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.453125" customWidth="1"/>
+    <col min="19" max="19" width="24.1796875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="26.81640625" customWidth="1"/>
+    <col min="21" max="21" width="27.26953125" customWidth="1"/>
+    <col min="22" max="22" width="7.1796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="14.453125" customWidth="1"/>
+    <col min="24" max="24" width="14.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="13" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -968,7 +969,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -1038,7 +1039,7 @@
       </c>
       <c r="X2" s="1"/>
     </row>
-    <row r="3" spans="1:24" s="9" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" s="9" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
         <v>53</v>
       </c>
@@ -1106,7 +1107,7 @@
       </c>
       <c r="X3" s="6"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1176,7 +1177,7 @@
       </c>
       <c r="X4" s="1"/>
     </row>
-    <row r="5" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>53</v>
       </c>
@@ -1246,7 +1247,7 @@
       </c>
       <c r="X5" s="1"/>
     </row>
-    <row r="6" spans="1:24" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" s="9" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>21</v>
       </c>
@@ -1316,7 +1317,7 @@
       </c>
       <c r="X6" s="6"/>
     </row>
-    <row r="7" spans="1:24" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
@@ -1384,7 +1385,7 @@
       </c>
       <c r="X7" s="1"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>44</v>
       </c>
@@ -1452,7 +1453,7 @@
       </c>
       <c r="X8" s="1"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
@@ -1520,7 +1521,7 @@
       </c>
       <c r="X9" s="1"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>53</v>
       </c>
@@ -1590,7 +1591,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>53</v>
       </c>
@@ -1656,7 +1657,7 @@
       </c>
       <c r="X11" s="1"/>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>53</v>
       </c>
@@ -1726,7 +1727,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>53</v>
       </c>
@@ -1798,7 +1799,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
@@ -1868,7 +1869,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
@@ -1938,7 +1939,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>53</v>
       </c>
@@ -2006,7 +2007,7 @@
       </c>
       <c r="X16" s="1"/>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>74</v>
       </c>
@@ -2074,7 +2075,7 @@
       </c>
       <c r="X17" s="1"/>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>74</v>
       </c>
@@ -2142,7 +2143,7 @@
       </c>
       <c r="X18" s="1"/>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>81</v>
       </c>
@@ -2212,7 +2213,7 @@
       </c>
       <c r="X19" s="1"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>81</v>
       </c>
@@ -2282,7 +2283,7 @@
       </c>
       <c r="X20" s="1"/>
     </row>
-    <row r="21" spans="1:24" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>90</v>
       </c>
@@ -2354,7 +2355,7 @@
       </c>
       <c r="X21" s="14"/>
     </row>
-    <row r="22" spans="1:24" s="17" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" s="17" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="14" t="s">
         <v>90</v>
       </c>
@@ -2426,7 +2427,7 @@
       </c>
       <c r="X22" s="14"/>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>90</v>
       </c>
@@ -2492,7 +2493,7 @@
       </c>
       <c r="X23" s="1"/>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>90</v>
       </c>

</xml_diff>